<commit_message>
feat: new bill info
</commit_message>
<xml_diff>
--- a/MuoiCu_Server/templates/Phieu_Sua_Chua.xlsx
+++ b/MuoiCu_Server/templates/Phieu_Sua_Chua.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t>Mã HEAD/Tên HEAD</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
   </si>
   <si>
     <t>Tên khách hàng: VÕ HOÀNG TRỌNG</t>
@@ -1619,16 +1616,14 @@
         <v>6</v>
       </c>
       <c r="AD6" s="30"/>
-      <c r="AE6" s="31" t="s">
-        <v>7</v>
-      </c>
+      <c r="AE6" s="31"/>
       <c r="AF6" s="15"/>
       <c r="AG6" s="15"/>
       <c r="AH6" s="2"/>
     </row>
     <row r="7" ht="28.5" customHeight="1">
       <c r="A7" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
@@ -1639,7 +1634,7 @@
       <c r="H7" s="33"/>
       <c r="I7" s="34"/>
       <c r="J7" s="35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K7" s="33"/>
       <c r="L7" s="33"/>
@@ -1655,7 +1650,7 @@
       <c r="V7" s="33"/>
       <c r="W7" s="34"/>
       <c r="X7" s="36" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Y7" s="37"/>
       <c r="Z7" s="37"/>
@@ -1693,7 +1688,7 @@
       <c r="V8" s="44"/>
       <c r="W8" s="45"/>
       <c r="X8" s="36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Y8" s="37"/>
       <c r="Z8" s="37"/>
@@ -1708,7 +1703,7 @@
     </row>
     <row r="9" ht="36.75" customHeight="1">
       <c r="A9" s="36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="47"/>
       <c r="C9" s="47"/>
@@ -1719,7 +1714,7 @@
       <c r="H9" s="47"/>
       <c r="I9" s="48"/>
       <c r="J9" s="36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K9" s="29"/>
       <c r="L9" s="29"/>
@@ -1735,7 +1730,7 @@
       <c r="V9" s="29"/>
       <c r="W9" s="30"/>
       <c r="X9" s="36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Y9" s="37"/>
       <c r="Z9" s="37"/>
@@ -1750,7 +1745,7 @@
     </row>
     <row r="10" ht="36.75" customHeight="1">
       <c r="A10" s="49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" s="50"/>
       <c r="C10" s="50"/>
@@ -1761,7 +1756,7 @@
       <c r="H10" s="51"/>
       <c r="I10" s="52"/>
       <c r="J10" s="36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K10" s="29"/>
       <c r="L10" s="29"/>
@@ -1777,7 +1772,7 @@
       <c r="V10" s="29"/>
       <c r="W10" s="30"/>
       <c r="X10" s="53" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Y10" s="54"/>
       <c r="Z10" s="54"/>
@@ -1792,7 +1787,7 @@
     </row>
     <row r="11" ht="36.75" customHeight="1">
       <c r="A11" s="49" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="47"/>
       <c r="C11" s="55"/>
@@ -1801,11 +1796,11 @@
       <c r="F11" s="55"/>
       <c r="G11" s="55"/>
       <c r="H11" s="51" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I11" s="30"/>
       <c r="J11" s="36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K11" s="29"/>
       <c r="L11" s="29"/>
@@ -1821,7 +1816,7 @@
       <c r="V11" s="29"/>
       <c r="W11" s="30"/>
       <c r="X11" s="53" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Y11" s="54"/>
       <c r="Z11" s="54"/>
@@ -1836,7 +1831,7 @@
     </row>
     <row r="12" ht="26.25" customHeight="1">
       <c r="A12" s="56" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="29"/>
       <c r="C12" s="29"/>
@@ -1848,7 +1843,7 @@
       <c r="I12" s="48"/>
       <c r="J12" s="57"/>
       <c r="K12" s="58" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L12" s="29"/>
       <c r="M12" s="29"/>
@@ -1869,7 +1864,7 @@
       <c r="AB12" s="29"/>
       <c r="AC12" s="30"/>
       <c r="AD12" s="56" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AE12" s="30"/>
       <c r="AF12" s="15"/>
@@ -1878,7 +1873,7 @@
     </row>
     <row r="13" ht="34.5" customHeight="1">
       <c r="A13" s="59" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="33"/>
@@ -1889,7 +1884,7 @@
       <c r="H13" s="33"/>
       <c r="I13" s="34"/>
       <c r="J13" s="60" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K13" s="33"/>
       <c r="L13" s="33"/>
@@ -1912,7 +1907,7 @@
       <c r="AC13" s="34"/>
       <c r="AD13" s="61"/>
       <c r="AE13" s="62" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AF13" s="15"/>
       <c r="AG13" s="15"/>
@@ -1925,7 +1920,7 @@
       <c r="AC14" s="64"/>
       <c r="AD14" s="61"/>
       <c r="AE14" s="65" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AF14" s="15"/>
       <c r="AG14" s="15"/>
@@ -1963,7 +1958,7 @@
       <c r="AC15" s="45"/>
       <c r="AD15" s="61"/>
       <c r="AE15" s="66" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AF15" s="15"/>
       <c r="AG15" s="15"/>
@@ -2007,7 +2002,7 @@
     </row>
     <row r="17" ht="31.5" customHeight="1">
       <c r="A17" s="68" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="29"/>
       <c r="C17" s="29"/>
@@ -2021,11 +2016,11 @@
       <c r="K17" s="29"/>
       <c r="L17" s="69"/>
       <c r="M17" s="70" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N17" s="30"/>
       <c r="O17" s="71" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P17" s="29"/>
       <c r="Q17" s="29"/>
@@ -2049,10 +2044,10 @@
     </row>
     <row r="18" ht="45.75" customHeight="1">
       <c r="A18" s="72" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="73" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" s="29"/>
       <c r="D18" s="29"/>
@@ -2060,30 +2055,30 @@
       <c r="F18" s="29"/>
       <c r="G18" s="30"/>
       <c r="H18" s="73" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I18" s="30"/>
       <c r="J18" s="74" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="75" t="s">
         <v>36</v>
       </c>
-      <c r="K18" s="75" t="s">
+      <c r="L18" s="76" t="s">
         <v>37</v>
       </c>
-      <c r="L18" s="76" t="s">
+      <c r="M18" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="M18" s="77" t="s">
+      <c r="N18" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="N18" s="77" t="s">
+      <c r="O18" s="73" t="s">
         <v>40</v>
-      </c>
-      <c r="O18" s="73" t="s">
-        <v>41</v>
       </c>
       <c r="P18" s="30"/>
       <c r="Q18" s="78" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="R18" s="29"/>
       <c r="S18" s="29"/>
@@ -2093,14 +2088,14 @@
       <c r="W18" s="29"/>
       <c r="X18" s="30"/>
       <c r="Y18" s="78" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Z18" s="29"/>
       <c r="AA18" s="29"/>
       <c r="AB18" s="29"/>
       <c r="AC18" s="30"/>
       <c r="AD18" s="78" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AE18" s="30"/>
       <c r="AF18" s="2"/>
@@ -2112,7 +2107,7 @@
         <v>1.0</v>
       </c>
       <c r="B19" s="79" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" s="80"/>
       <c r="D19" s="80"/>
@@ -2120,7 +2115,7 @@
       <c r="F19" s="80"/>
       <c r="G19" s="81"/>
       <c r="H19" s="82" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I19" s="30"/>
       <c r="J19" s="82"/>
@@ -2846,7 +2841,7 @@
         <v>20.0</v>
       </c>
       <c r="B38" s="56" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C38" s="29"/>
       <c r="D38" s="29"/>
@@ -2961,7 +2956,7 @@
     </row>
     <row r="41" ht="24.0" customHeight="1">
       <c r="A41" s="103" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B41" s="104"/>
       <c r="C41" s="104"/>
@@ -2970,17 +2965,17 @@
       <c r="F41" s="104"/>
       <c r="G41" s="104"/>
       <c r="H41" s="105" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I41" s="106"/>
       <c r="J41" s="56" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K41" s="29"/>
       <c r="L41" s="107"/>
       <c r="M41" s="108"/>
       <c r="N41" s="109" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O41" s="110"/>
       <c r="P41" s="110"/>
@@ -3018,7 +3013,7 @@
       <c r="L42" s="114"/>
       <c r="M42" s="114"/>
       <c r="N42" s="115" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O42" s="33"/>
       <c r="P42" s="33"/>
@@ -3034,12 +3029,12 @@
       <c r="Z42" s="33"/>
       <c r="AA42" s="34"/>
       <c r="AB42" s="116" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AC42" s="33"/>
       <c r="AD42" s="34"/>
       <c r="AE42" s="117" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AF42" s="2"/>
       <c r="AG42" s="2"/>
@@ -3047,7 +3042,7 @@
     </row>
     <row r="43" ht="19.5" customHeight="1">
       <c r="A43" s="118" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B43" s="27"/>
       <c r="C43" s="27"/>
@@ -3098,7 +3093,7 @@
       <c r="L44" s="124"/>
       <c r="M44" s="114"/>
       <c r="N44" s="125" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O44" s="33"/>
       <c r="P44" s="33"/>
@@ -3150,7 +3145,7 @@
     </row>
     <row r="46" ht="19.5" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -3247,14 +3242,14 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="135"/>
       <c r="D49" s="135"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -3776,7 +3771,7 @@
     </row>
     <row r="65" ht="43.5" customHeight="1">
       <c r="A65" s="144" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AF65" s="2"/>
       <c r="AG65" s="2"/>

</xml_diff>